<commit_message>
Questions for SQL updated
</commit_message>
<xml_diff>
--- a/Assignment Difference.xlsx
+++ b/Assignment Difference.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QSpider\1. SQL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C945730F-539B-4411-BEF8-6F1FC98CD9D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31AAA896-DAB0-4A7A-AF75-7551E9D1CDD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E787B147-5774-42C4-9CE4-48E9852B8AB5}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="179">
   <si>
     <t>Fixed length memory allocation</t>
   </si>
@@ -325,9 +325,6 @@
   </si>
   <si>
     <t>Eliminates duplicate rows from the output of a SELECT statement.</t>
-  </si>
-  <si>
-    <t>Type</t>
   </si>
   <si>
     <t>SQL Keyword</t>
@@ -1390,7 +1387,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>28</v>
@@ -1407,7 +1404,7 @@
         <v>36</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>94</v>
@@ -1426,46 +1423,46 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B44" s="2" t="s">
-        <v>97</v>
+        <v>56</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B45" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B46" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="D46" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B47" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="D47" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
@@ -1473,10 +1470,10 @@
         <v>3</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.35">
@@ -1484,10 +1481,10 @@
         <v>80</v>
       </c>
       <c r="C49" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.35">
@@ -1495,10 +1492,10 @@
         <v>28</v>
       </c>
       <c r="C51" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D51" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="52" spans="2:4" ht="43.5" x14ac:dyDescent="0.35">
@@ -1506,43 +1503,43 @@
         <v>36</v>
       </c>
       <c r="C52" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B53" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C53" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B54" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="55" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B55" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.35">
@@ -1550,10 +1547,10 @@
         <v>19</v>
       </c>
       <c r="C56" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.35">
@@ -1561,10 +1558,10 @@
         <v>28</v>
       </c>
       <c r="C58" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D58" s="3" t="s">
         <v>129</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="59" spans="2:4" ht="29" x14ac:dyDescent="0.35">
@@ -1572,76 +1569,76 @@
         <v>36</v>
       </c>
       <c r="C59" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="60" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B60" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C60" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D60" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B61" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C61" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B62" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C62" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>146</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B63" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="D63" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="64" spans="2:4" ht="58" x14ac:dyDescent="0.35">
       <c r="B64" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="65" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B65" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="D65" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.35">
@@ -1649,30 +1646,30 @@
         <v>19</v>
       </c>
       <c r="C66" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="67" spans="2:4" ht="6.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="68" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B68" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C68" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="D68" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="69" spans="2:4" ht="101.5" x14ac:dyDescent="0.35">
       <c r="B69" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.35">
@@ -1680,10 +1677,10 @@
         <v>28</v>
       </c>
       <c r="C71" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D71" s="3" t="s">
         <v>158</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="72" spans="2:4" ht="29" x14ac:dyDescent="0.35">
@@ -1691,32 +1688,32 @@
         <v>36</v>
       </c>
       <c r="C72" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D72" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="73" spans="2:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B73" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C73" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="74" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B74" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="D74" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.35">
@@ -1724,10 +1721,10 @@
         <v>28</v>
       </c>
       <c r="C76" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D76" s="3" t="s">
         <v>168</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="77" spans="2:4" ht="43.5" x14ac:dyDescent="0.35">
@@ -1735,43 +1732,43 @@
         <v>36</v>
       </c>
       <c r="C77" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="78" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B78" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="79" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B79" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="D79" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="80" spans="2:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B80" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C80" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="D80" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>